<commit_message>
30 noviembre de 2020 v1
</commit_message>
<xml_diff>
--- a/_downloads/be2fbcfffa0bffb8ba54a662e9d97b81/Ejemplos valoración de opciones por AB y BS.xlsx
+++ b/_downloads/be2fbcfffa0bffb8ba54a662e9d97b81/Ejemplos valoración de opciones por AB y BS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\DERIVADOS FINANCIEROS\CLASES\Opciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E452EA97-5E58-482F-BB07-BFC10385C315}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5442B786-FBE5-46F0-92AA-2426B5A13303}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{04782C71-9EF5-45E7-9F04-DD1E48186E05}"/>
   </bookViews>
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="41">
   <si>
     <t>Volatilidad</t>
   </si>
@@ -366,6 +366,12 @@
   <si>
     <t>Divisas</t>
   </si>
+  <si>
+    <t>Call Americana:</t>
+  </si>
+  <si>
+    <t>Put Americana:</t>
+  </si>
 </sst>
 </file>
 
@@ -464,21 +470,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="6" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="8" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="6" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="8" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="8" fontId="5" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -487,6 +484,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -519,8 +525,8 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>177703</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 1">
@@ -726,7 +732,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 1">
@@ -887,8 +893,8 @@
       <xdr:row>13</xdr:row>
       <xdr:rowOff>27606</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 2">
@@ -1066,7 +1072,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 2">
@@ -1220,8 +1226,8 @@
       <xdr:row>15</xdr:row>
       <xdr:rowOff>64987</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="CuadroTexto 7">
@@ -1454,7 +1460,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="CuadroTexto 7">
@@ -1608,8 +1614,8 @@
       <xdr:row>17</xdr:row>
       <xdr:rowOff>20191</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="CuadroTexto 9">
@@ -1768,7 +1774,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="CuadroTexto 9">
@@ -1922,8 +1928,8 @@
       <xdr:row>22</xdr:row>
       <xdr:rowOff>177703</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="CuadroTexto 5">
@@ -2129,7 +2135,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="CuadroTexto 5">
@@ -2290,8 +2296,8 @@
       <xdr:row>25</xdr:row>
       <xdr:rowOff>27606</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -2469,7 +2475,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -2623,8 +2629,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>64987</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="CuadroTexto 7">
@@ -2857,7 +2863,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="CuadroTexto 7">
@@ -3011,8 +3017,8 @@
       <xdr:row>29</xdr:row>
       <xdr:rowOff>20191</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="CuadroTexto 9">
@@ -3171,7 +3177,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="CuadroTexto 9">
@@ -3413,8 +3419,8 @@
       <xdr:row>7</xdr:row>
       <xdr:rowOff>39675</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="126" name="CuadroTexto 11">
@@ -3699,7 +3705,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="126" name="CuadroTexto 11">
@@ -3871,8 +3877,8 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>177703</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 1">
@@ -4078,7 +4084,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 1">
@@ -4239,8 +4245,8 @@
       <xdr:row>13</xdr:row>
       <xdr:rowOff>27606</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 2">
@@ -4418,7 +4424,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 2">
@@ -4572,8 +4578,8 @@
       <xdr:row>15</xdr:row>
       <xdr:rowOff>64987</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="CuadroTexto 7">
@@ -4806,7 +4812,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="CuadroTexto 7">
@@ -4960,8 +4966,8 @@
       <xdr:row>17</xdr:row>
       <xdr:rowOff>20191</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="CuadroTexto 9">
@@ -5120,7 +5126,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="CuadroTexto 9">
@@ -5274,8 +5280,8 @@
       <xdr:row>22</xdr:row>
       <xdr:rowOff>177703</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="CuadroTexto 5">
@@ -5481,7 +5487,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="CuadroTexto 5">
@@ -5642,8 +5648,8 @@
       <xdr:row>25</xdr:row>
       <xdr:rowOff>27606</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -5821,7 +5827,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -5975,8 +5981,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>64987</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="CuadroTexto 7">
@@ -6209,7 +6215,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="CuadroTexto 7">
@@ -6363,8 +6369,8 @@
       <xdr:row>29</xdr:row>
       <xdr:rowOff>20191</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="CuadroTexto 9">
@@ -6523,7 +6529,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="CuadroTexto 9">
@@ -6765,8 +6771,8 @@
       <xdr:row>7</xdr:row>
       <xdr:rowOff>30991</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="14" name="CuadroTexto 11">
@@ -7051,7 +7057,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="14" name="CuadroTexto 11">
@@ -7223,8 +7229,8 @@
       <xdr:row>9</xdr:row>
       <xdr:rowOff>190735</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="CuadroTexto 14">
@@ -7576,7 +7582,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="CuadroTexto 14">
@@ -7759,8 +7765,8 @@
       <xdr:row>11</xdr:row>
       <xdr:rowOff>174330</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="13" name="CuadroTexto 17">
@@ -7987,7 +7993,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="13" name="CuadroTexto 17">
@@ -8144,8 +8150,8 @@
       <xdr:row>17</xdr:row>
       <xdr:rowOff>44506</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="14" name="CuadroTexto 12">
@@ -8447,7 +8453,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="14" name="CuadroTexto 12">
@@ -8597,8 +8603,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>27204</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="15" name="CuadroTexto 15">
@@ -8911,7 +8917,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="15" name="CuadroTexto 15">
@@ -9066,8 +9072,8 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>177703</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 1">
@@ -9273,7 +9279,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 1">
@@ -9434,8 +9440,8 @@
       <xdr:row>13</xdr:row>
       <xdr:rowOff>27606</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 2">
@@ -9613,7 +9619,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 2">
@@ -9767,8 +9773,8 @@
       <xdr:row>15</xdr:row>
       <xdr:rowOff>169187</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="CuadroTexto 7">
@@ -10069,7 +10075,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="CuadroTexto 7">
@@ -10263,8 +10269,8 @@
       <xdr:row>17</xdr:row>
       <xdr:rowOff>123605</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="CuadroTexto 9">
@@ -10423,7 +10429,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="CuadroTexto 9">
@@ -10577,8 +10583,8 @@
       <xdr:row>22</xdr:row>
       <xdr:rowOff>177703</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="CuadroTexto 5">
@@ -10784,7 +10790,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="CuadroTexto 5">
@@ -10945,8 +10951,8 @@
       <xdr:row>25</xdr:row>
       <xdr:rowOff>27606</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -11124,7 +11130,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -11278,8 +11284,8 @@
       <xdr:row>30</xdr:row>
       <xdr:rowOff>14748</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="CuadroTexto 9">
@@ -11438,7 +11444,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="CuadroTexto 9">
@@ -11592,8 +11598,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>169187</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="CuadroTexto 7">
@@ -11894,7 +11900,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="CuadroTexto 7">
@@ -12176,8 +12182,8 @@
       <xdr:row>7</xdr:row>
       <xdr:rowOff>58205</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="15" name="CuadroTexto 11">
@@ -12462,7 +12468,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="15" name="CuadroTexto 11">
@@ -12634,8 +12640,8 @@
       <xdr:row>10</xdr:row>
       <xdr:rowOff>177703</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 1">
@@ -12841,7 +12847,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="2" name="CuadroTexto 1">
@@ -13002,8 +13008,8 @@
       <xdr:row>13</xdr:row>
       <xdr:rowOff>27606</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 2">
@@ -13181,7 +13187,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 2">
@@ -13335,8 +13341,8 @@
       <xdr:row>15</xdr:row>
       <xdr:rowOff>169187</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="CuadroTexto 7">
@@ -13637,7 +13643,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="4" name="CuadroTexto 7">
@@ -13831,8 +13837,8 @@
       <xdr:row>17</xdr:row>
       <xdr:rowOff>123605</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="CuadroTexto 9">
@@ -13991,7 +13997,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="CuadroTexto 9">
@@ -14145,8 +14151,8 @@
       <xdr:row>22</xdr:row>
       <xdr:rowOff>177703</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="CuadroTexto 5">
@@ -14352,7 +14358,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="CuadroTexto 5">
@@ -14513,8 +14519,8 @@
       <xdr:row>25</xdr:row>
       <xdr:rowOff>27606</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -14692,7 +14698,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -14846,8 +14852,8 @@
       <xdr:row>30</xdr:row>
       <xdr:rowOff>14748</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="CuadroTexto 9">
@@ -15006,7 +15012,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="CuadroTexto 9">
@@ -15160,8 +15166,8 @@
       <xdr:row>27</xdr:row>
       <xdr:rowOff>169187</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="CuadroTexto 7">
@@ -15462,7 +15468,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="CuadroTexto 7">
@@ -15656,8 +15662,8 @@
       <xdr:row>7</xdr:row>
       <xdr:rowOff>58205</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="CuadroTexto 11">
@@ -15942,7 +15948,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="12" name="CuadroTexto 11">
@@ -16202,8 +16208,8 @@
       <xdr:row>11</xdr:row>
       <xdr:rowOff>174330</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 17">
@@ -16430,7 +16436,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="3" name="CuadroTexto 17">
@@ -16587,8 +16593,8 @@
       <xdr:row>9</xdr:row>
       <xdr:rowOff>201622</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="CuadroTexto 8">
@@ -16975,7 +16981,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="6" name="CuadroTexto 8">
@@ -17162,8 +17168,8 @@
       <xdr:row>17</xdr:row>
       <xdr:rowOff>4353</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -17525,7 +17531,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="7" name="CuadroTexto 6">
@@ -17679,8 +17685,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>26125</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="CuadroTexto 7">
@@ -18053,7 +18059,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="8" name="CuadroTexto 7">
@@ -18513,11 +18519,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:12" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -18572,26 +18578,26 @@
       <c r="B7" s="3"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="4">
         <f>6/12</f>
         <v>0.5</v>
       </c>
@@ -18600,14 +18606,14 @@
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="5"/>
-      <c r="J10" s="5" t="s">
+      <c r="G10" s="16"/>
+      <c r="J10" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="K10" s="5"/>
+      <c r="K10" s="16"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
@@ -18619,11 +18625,11 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G12" s="7">
+      <c r="G12" s="5">
         <f>+F13*u</f>
         <v>1151.9099101689089</v>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="5">
         <f>+J13*u</f>
         <v>1151.9099101689089</v>
       </c>
@@ -18636,37 +18642,37 @@
         <f>1/B11</f>
         <v>0.86812344539458486</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="9">
         <f>+MAX(G12-K,0)</f>
         <v>101.90991016890894</v>
       </c>
-      <c r="J13" s="8">
+      <c r="J13" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="9">
         <f>+MAX(K-K12,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F14" s="13">
+      <c r="F14" s="10">
         <f>+(G13*p+G15*q)*EXP(-risk*deltaT)</f>
         <v>55.05501951406594</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="5">
         <f>+F13*d</f>
         <v>868.12344539458491</v>
       </c>
-      <c r="J14" s="13">
+      <c r="J14" s="10">
         <f>+(K13*p+K15*q)*EXP(-risk*deltaT)</f>
         <v>79.130427143815226</v>
       </c>
-      <c r="K14" s="7">
+      <c r="K14" s="5">
         <f>+J13*d</f>
         <v>868.12344539458491</v>
       </c>
@@ -18679,11 +18685,11 @@
         <f>+(EXP(risk*deltaT)-d)/(u-d)</f>
         <v>0.55390828894833921</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="9">
         <f>+MAX(G14-K,0)</f>
         <v>0</v>
       </c>
-      <c r="K15" s="12">
+      <c r="K15" s="9">
         <f>+MAX(K-K14,0)</f>
         <v>181.87655460541509</v>
       </c>
@@ -18696,34 +18702,34 @@
         <f>1-p</f>
         <v>0.44609171105166079</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J17" s="6" t="s">
+      <c r="J17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K17" s="6" t="s">
+      <c r="K17" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -18745,16 +18751,16 @@
         <f>+EXP(vol*SQRT(B21))</f>
         <v>1.1051709180756477</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="J23" s="5" t="s">
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="J23" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
@@ -18764,29 +18770,29 @@
         <f>1/B23</f>
         <v>0.90483741803595952</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="5">
         <f>+G26*B23</f>
         <v>1221.4027581601699</v>
       </c>
-      <c r="L25" s="7">
+      <c r="L25" s="5">
         <f>+K26*B23</f>
         <v>1221.4027581601699</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G26" s="7">
+      <c r="G26" s="5">
         <f>+F27*B23</f>
         <v>1105.1709180756477</v>
       </c>
-      <c r="H26" s="12">
+      <c r="H26" s="9">
         <f>+MAX(H25-K,0)</f>
         <v>171.40275816016992</v>
       </c>
-      <c r="K26" s="7">
+      <c r="K26" s="5">
         <f>+J27*B23</f>
         <v>1105.1709180756477</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L26" s="9">
         <f>+MAX(K-L25,0)</f>
         <v>0</v>
       </c>
@@ -18799,53 +18805,53 @@
         <f>+(EXP(risk*B21)-B25)/(B23-B25)</f>
         <v>0.53780837195641396</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="G27" s="12">
+      <c r="G27" s="9">
         <f>+(H26*$B$27+H28*$B$29)*EXP(-risk*$B$21)</f>
         <v>91.036737128570735</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="6">
         <f>+G28*B23</f>
         <v>1000.0000000000001</v>
       </c>
-      <c r="J27" s="8">
+      <c r="J27" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="K27" s="12">
+      <c r="K27" s="9">
         <f>+(L26*$B$27+L28*$B$29)*EXP(-risk*$B$21)</f>
         <v>22.82250957149849</v>
       </c>
-      <c r="L27" s="8">
+      <c r="L27" s="6">
         <f>+K28*B23</f>
         <v>1000.0000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F28" s="13">
+      <c r="F28" s="10">
         <f>+(G27*$B$27+G29*$B$29)*EXP(-risk*$B$21)</f>
         <v>48.35212452807751</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="5">
         <f>+F27*B25</f>
         <v>904.83741803595956</v>
       </c>
-      <c r="H28" s="12">
+      <c r="H28" s="9">
         <f>+MAX(H27-K,0)</f>
         <v>0</v>
       </c>
-      <c r="J28" s="13">
+      <c r="J28" s="10">
         <f>+(K27*$B$27+K29*$B$29)*EXP(-risk*$B$21)</f>
         <v>72.427532157826704</v>
       </c>
-      <c r="K28" s="7">
+      <c r="K28" s="5">
         <f>+J27*B25</f>
         <v>904.83741803595956</v>
       </c>
-      <c r="L28" s="12">
+      <c r="L28" s="9">
         <f>+MAX(K-L27,0)</f>
         <v>49.999999999999886</v>
       </c>
@@ -18858,96 +18864,96 @@
         <f>1-B27</f>
         <v>0.46219162804358604</v>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="9">
         <f>+(H28*$B$27+H30*$B$29)*EXP(-risk*$B$21)</f>
         <v>0</v>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="5">
         <f>+G28*B25</f>
         <v>818.73075307798183</v>
       </c>
-      <c r="K29" s="12">
+      <c r="K29" s="9">
         <f>+(L28*$B$27+L30*$B$29)*EXP(-risk*$B$21)</f>
         <v>132.11927248261588</v>
       </c>
-      <c r="L29" s="7">
+      <c r="L29" s="5">
         <f>+K28*B25</f>
         <v>818.73075307798183</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="H30" s="12">
+      <c r="H30" s="9">
         <f>+MAX(H29-K,0)</f>
         <v>0</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L30" s="9">
         <f>+MAX(K-L29,0)</f>
         <v>231.26924692201817</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F32" s="6" t="s">
+      <c r="F32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="G32" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H32" s="6" t="s">
+      <c r="H32" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J32" s="6" t="s">
+      <c r="J32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K32" s="6" t="s">
+      <c r="K32" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="L32" s="6" t="s">
+      <c r="L32" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="D33" s="9"/>
+      <c r="D33" s="7"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15"/>
+      <c r="L35" s="15"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="H37" s="5" t="s">
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="H37" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="11" t="s">
+      <c r="A58" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B58" s="11"/>
-      <c r="C58" s="11"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="8"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B59" s="13">
+      <c r="B59" s="10">
         <v>45.813136870375402</v>
       </c>
     </row>
@@ -18955,7 +18961,7 @@
       <c r="A60" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B60" s="13">
+      <c r="B60" s="10">
         <v>69.8885445001075</v>
       </c>
     </row>
@@ -19001,11 +19007,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:12" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -19060,26 +19066,26 @@
       <c r="B7" s="3"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="4">
         <f>6/12</f>
         <v>0.5</v>
       </c>
@@ -19088,14 +19094,14 @@
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F10" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" s="5"/>
-      <c r="J10" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="K10" s="5"/>
+      <c r="F10" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="16"/>
+      <c r="J10" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="K10" s="16"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
@@ -19107,11 +19113,11 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G12" s="7">
+      <c r="G12" s="5">
         <f>+F13*u</f>
         <v>1151.9099101689089</v>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="5">
         <f>+J13*u</f>
         <v>1151.9099101689089</v>
       </c>
@@ -19124,37 +19130,37 @@
         <f>1/B11</f>
         <v>0.86812344539458486</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="9">
         <f>+MAX(G12-K,0)</f>
         <v>101.90991016890894</v>
       </c>
-      <c r="J13" s="8">
+      <c r="J13" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="9">
         <f>+MAX(K-K12,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F14" s="13">
+      <c r="F14" s="10">
         <f>+MAX((G13*p+G15*q)*EXP(-risk*deltaT),MAX(F13-K,0))</f>
         <v>55.05501951406594</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="5">
         <f>+F13*d</f>
         <v>868.12344539458491</v>
       </c>
-      <c r="J14" s="13">
+      <c r="J14" s="10">
         <f>+MAX((K13*p+K15*q)*EXP(-risk*deltaT),MAX(K-J13,0))</f>
         <v>79.130427143815226</v>
       </c>
-      <c r="K14" s="7">
+      <c r="K14" s="5">
         <f>+J13*d</f>
         <v>868.12344539458491</v>
       </c>
@@ -19167,11 +19173,11 @@
         <f>+(EXP(risk*deltaT)-d)/(u-d)</f>
         <v>0.55390828894833921</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="9">
         <f>+MAX(G14-K,0)</f>
         <v>0</v>
       </c>
-      <c r="K15" s="12">
+      <c r="K15" s="9">
         <f>+MAX(K-K14,0)</f>
         <v>181.87655460541509</v>
       </c>
@@ -19184,34 +19190,34 @@
         <f>1-p</f>
         <v>0.44609171105166079</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J17" s="6" t="s">
+      <c r="J17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K17" s="6" t="s">
+      <c r="K17" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -19224,7 +19230,7 @@
       <c r="C21" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="I21" s="14"/>
+      <c r="I21" s="11"/>
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
@@ -19234,16 +19240,16 @@
         <f>+EXP(vol*SQRT(B21))</f>
         <v>1.1051709180756477</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="J23" s="5" t="s">
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="J23" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
@@ -19253,29 +19259,29 @@
         <f>1/B23</f>
         <v>0.90483741803595952</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="5">
         <f>+G26*B23</f>
         <v>1221.4027581601699</v>
       </c>
-      <c r="L25" s="7">
+      <c r="L25" s="5">
         <f>+K26*B23</f>
         <v>1221.4027581601699</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G26" s="7">
+      <c r="G26" s="5">
         <f>+F27*B23</f>
         <v>1105.1709180756477</v>
       </c>
-      <c r="H26" s="12">
+      <c r="H26" s="9">
         <f>+MAX(H25-K,0)</f>
         <v>171.40275816016992</v>
       </c>
-      <c r="K26" s="7">
+      <c r="K26" s="5">
         <f>+J27*B23</f>
         <v>1105.1709180756477</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L26" s="9">
         <f>+MAX(K-L25,0)</f>
         <v>0</v>
       </c>
@@ -19288,53 +19294,53 @@
         <f>+(EXP(risk*B21)-B25)/(B23-B25)</f>
         <v>0.53780837195641396</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="G27" s="12">
+      <c r="G27" s="9">
         <f>+MAX((H26*$B$27+H28*$B$29)*EXP(-risk*$B$21),MAX(G26-K,0))</f>
         <v>91.036737128570735</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="6">
         <f>+G28*B23</f>
         <v>1000.0000000000001</v>
       </c>
-      <c r="J27" s="8">
+      <c r="J27" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="K27" s="12">
+      <c r="K27" s="9">
         <f>+MAX((L26*$B$27+L28*$B$29)*EXP(-risk*$B$21),MAX(K-K26,0))</f>
         <v>22.82250957149849</v>
       </c>
-      <c r="L27" s="8">
+      <c r="L27" s="6">
         <f>+K28*B23</f>
         <v>1000.0000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F28" s="13">
+      <c r="F28" s="10">
         <f>+MAX((G27*$B$27+G29*$B$29)*EXP(-risk*$B$21),MAX(F27-K,0))</f>
         <v>48.35212452807751</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="5">
         <f>+F27*B25</f>
         <v>904.83741803595956</v>
       </c>
-      <c r="H28" s="12">
+      <c r="H28" s="9">
         <f>+MAX(H27-K,0)</f>
         <v>0</v>
       </c>
-      <c r="J28" s="13">
+      <c r="J28" s="10">
         <f>+MAX((K27*$B$27+K29*$B$29)*EXP(-risk*$B$21),MAX(K-J27,0))</f>
         <v>78.381153267503294</v>
       </c>
-      <c r="K28" s="7">
+      <c r="K28" s="5">
         <f>+J27*B25</f>
         <v>904.83741803595956</v>
       </c>
-      <c r="L28" s="12">
+      <c r="L28" s="9">
         <f>+MAX(K-L27,0)</f>
         <v>49.999999999999886</v>
       </c>
@@ -19347,96 +19353,96 @@
         <f>1-B27</f>
         <v>0.46219162804358604</v>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="9">
         <f>+MAX((H28*$B$27+H30*$B$29)*EXP(-risk*$B$21),MAX(G28-K,0))</f>
         <v>0</v>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="5">
         <f>+G28*B25</f>
         <v>818.73075307798183</v>
       </c>
-      <c r="K29" s="12">
+      <c r="K29" s="9">
         <f>+MAX((L28*$B$27+L30*$B$29)*EXP(-risk*$B$21),MAX(K-K28,0))</f>
         <v>145.16258196404044</v>
       </c>
-      <c r="L29" s="7">
+      <c r="L29" s="5">
         <f>+K28*B25</f>
         <v>818.73075307798183</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="H30" s="12">
+      <c r="H30" s="9">
         <f>+MAX(H29-K,0)</f>
         <v>0</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L30" s="9">
         <f>+MAX(K-L29,0)</f>
         <v>231.26924692201817</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F32" s="6" t="s">
+      <c r="F32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="G32" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H32" s="6" t="s">
+      <c r="H32" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J32" s="6" t="s">
+      <c r="J32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K32" s="6" t="s">
+      <c r="K32" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="L32" s="6" t="s">
+      <c r="L32" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="D33" s="9"/>
+      <c r="D33" s="7"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15"/>
+      <c r="L35" s="15"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="H37" s="5" t="s">
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="H37" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="11" t="s">
+      <c r="A58" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="B58" s="11"/>
-      <c r="C58" s="11"/>
+      <c r="B58" s="8"/>
+      <c r="C58" s="8"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B59" s="13">
+      <c r="B59" s="10">
         <v>45.813136870375402</v>
       </c>
     </row>
@@ -19444,7 +19450,7 @@
       <c r="A60" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B60" s="13">
+      <c r="B60" s="10">
         <v>74.365645023472894</v>
       </c>
     </row>
@@ -19490,11 +19496,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:3" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -19594,7 +19600,7 @@
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="12">
         <f>+S*B14-K*EXP(-risk*T/12)*B15</f>
         <v>45.816801675400086</v>
       </c>
@@ -19624,7 +19630,7 @@
       <c r="A23" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="12">
         <f>+K*EXP(-risk*T/12)*B21-S*B20</f>
         <v>69.892209305149322</v>
       </c>
@@ -19659,11 +19665,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:12" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -19715,7 +19721,7 @@
       </c>
     </row>
     <row r="7" spans="1:12" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="13" t="s">
         <v>37</v>
       </c>
       <c r="B7" s="3">
@@ -19726,26 +19732,26 @@
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="4">
         <f>6/12</f>
         <v>0.5</v>
       </c>
@@ -19754,14 +19760,14 @@
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F10" s="5" t="s">
+      <c r="F10" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="5"/>
-      <c r="J10" s="5" t="s">
+      <c r="G10" s="16"/>
+      <c r="J10" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="K10" s="5"/>
+      <c r="K10" s="16"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
@@ -19773,11 +19779,11 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G12" s="7">
+      <c r="G12" s="5">
         <f>+F13*u</f>
         <v>1151.9099101689089</v>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="5">
         <f>+J13*u</f>
         <v>1151.9099101689089</v>
       </c>
@@ -19790,37 +19796,37 @@
         <f>1/B11</f>
         <v>0.86812344539458486</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="9">
         <f>+MAX(G12-K,0)</f>
         <v>101.90991016890894</v>
       </c>
-      <c r="J13" s="8">
+      <c r="J13" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="9">
         <f>+MAX(K-K12,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F14" s="13">
+      <c r="F14" s="10">
         <f>+(G13*p+G15*q)*EXP(-risk*deltaT)</f>
         <v>51.481838003825906</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="5">
         <f>+F13*d</f>
         <v>868.12344539458491</v>
       </c>
-      <c r="J14" s="13">
+      <c r="J14" s="10">
         <f>+(K13*p+K15*q)*EXP(-risk*deltaT)</f>
         <v>85.50741188440719</v>
       </c>
-      <c r="K14" s="7">
+      <c r="K14" s="5">
         <f>+J13*d</f>
         <v>868.12344539458491</v>
       </c>
@@ -19833,11 +19839,11 @@
         <f>+(EXP((risk-rf)*deltaT)-d)/(u-d)</f>
         <v>0.51795852680297783</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="9">
         <f>+MAX(G14-K,0)</f>
         <v>0</v>
       </c>
-      <c r="K15" s="12">
+      <c r="K15" s="9">
         <f>+MAX(K-K14,0)</f>
         <v>181.87655460541509</v>
       </c>
@@ -19850,34 +19856,34 @@
         <f>1-p</f>
         <v>0.48204147319702217</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J17" s="6" t="s">
+      <c r="J17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K17" s="6" t="s">
+      <c r="K17" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -19899,16 +19905,16 @@
         <f>+EXP(vol*SQRT(B21))</f>
         <v>1.1051709180756477</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="J23" s="5" t="s">
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="J23" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
@@ -19918,29 +19924,29 @@
         <f>1/B23</f>
         <v>0.90483741803595952</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="5">
         <f>+G26*B23</f>
         <v>1221.4027581601699</v>
       </c>
-      <c r="L25" s="7">
+      <c r="L25" s="5">
         <f>+K26*B23</f>
         <v>1221.4027581601699</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G26" s="7">
+      <c r="G26" s="5">
         <f>+F27*B23</f>
         <v>1105.1709180756477</v>
       </c>
-      <c r="H26" s="12">
+      <c r="H26" s="9">
         <f>+MAX(H25-K,0)</f>
         <v>171.40275816016992</v>
       </c>
-      <c r="K26" s="7">
+      <c r="K26" s="5">
         <f>+J27*B23</f>
         <v>1105.1709180756477</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L26" s="9">
         <f>+MAX(K-L25,0)</f>
         <v>0</v>
       </c>
@@ -19953,53 +19959,53 @@
         <f>+(EXP((risk-rf)*B21)-B25)/(B23-B25)</f>
         <v>0.51259912789538553</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="G27" s="12">
+      <c r="G27" s="9">
         <f>+(H26*$B$27+H28*$B$29)*EXP(-risk*$B$21)</f>
         <v>86.769478669121128</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="6">
         <f>+G28*B23</f>
         <v>1000.0000000000001</v>
       </c>
-      <c r="J27" s="8">
+      <c r="J27" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="K27" s="12">
+      <c r="K27" s="9">
         <f>+(L26*$B$27+L28*$B$29)*EXP(-risk*$B$21)</f>
         <v>24.067314061593681</v>
       </c>
-      <c r="L27" s="8">
+      <c r="L27" s="6">
         <f>+K28*B23</f>
         <v>1000.0000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F28" s="13">
+      <c r="F28" s="10">
         <f>+(G27*$B$27+G29*$B$29)*EXP(-risk*$B$21)</f>
         <v>43.925445012241468</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="5">
         <f>+F27*B25</f>
         <v>904.83741803595956</v>
       </c>
-      <c r="H28" s="12">
+      <c r="H28" s="9">
         <f>+MAX(H27-K,0)</f>
         <v>0</v>
       </c>
-      <c r="J28" s="13">
+      <c r="J28" s="10">
         <f>+(K27*$B$27+K29*$B$29)*EXP(-risk*$B$21)</f>
         <v>77.95101889282283</v>
       </c>
-      <c r="K28" s="7">
+      <c r="K28" s="5">
         <f>+J27*B25</f>
         <v>904.83741803595956</v>
       </c>
-      <c r="L28" s="12">
+      <c r="L28" s="9">
         <f>+MAX(K-L27,0)</f>
         <v>49.999999999999886</v>
       </c>
@@ -20012,96 +20018,96 @@
         <f>1-B27</f>
         <v>0.48740087210461447</v>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="9">
         <f>+(H28*$B$27+H30*$B$29)*EXP(-risk*$B$21)</f>
         <v>0</v>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="5">
         <f>+G28*B25</f>
         <v>818.73075307798183</v>
       </c>
-      <c r="K29" s="12">
+      <c r="K29" s="9">
         <f>+(L28*$B$27+L30*$B$29)*EXP(-risk*$B$21)</f>
         <v>136.63216793230993</v>
       </c>
-      <c r="L29" s="7">
+      <c r="L29" s="5">
         <f>+K28*B25</f>
         <v>818.73075307798183</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="H30" s="12">
+      <c r="H30" s="9">
         <f>+MAX(H29-K,0)</f>
         <v>0</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L30" s="9">
         <f>+MAX(K-L29,0)</f>
         <v>231.26924692201817</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F32" s="6" t="s">
+      <c r="F32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="G32" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H32" s="6" t="s">
+      <c r="H32" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J32" s="6" t="s">
+      <c r="J32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K32" s="6" t="s">
+      <c r="K32" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="L32" s="6" t="s">
+      <c r="L32" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="D33" s="9"/>
+      <c r="D33" s="7"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15"/>
+      <c r="L35" s="15"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="H37" s="5" t="s">
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="H37" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="10" t="s">
+      <c r="A58" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
+      <c r="B58" s="15"/>
+      <c r="C58" s="15"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B59" s="13">
+      <c r="B59" s="10">
         <v>41.364694755898398</v>
       </c>
     </row>
@@ -20109,7 +20115,7 @@
       <c r="A60" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B60" s="13">
+      <c r="B60" s="10">
         <v>75.390268636498305</v>
       </c>
     </row>
@@ -20156,11 +20162,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:12" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -20212,7 +20218,7 @@
       </c>
     </row>
     <row r="7" spans="1:12" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="13" t="s">
         <v>37</v>
       </c>
       <c r="B7" s="3">
@@ -20223,26 +20229,26 @@
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="10"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+      <c r="G8" s="15"/>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="6">
+      <c r="B9" s="4">
         <f>6/12</f>
         <v>0.5</v>
       </c>
@@ -20251,14 +20257,14 @@
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F10" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G10" s="5"/>
-      <c r="J10" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="K10" s="5"/>
+      <c r="F10" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="16"/>
+      <c r="J10" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="K10" s="16"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
@@ -20270,11 +20276,11 @@
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G12" s="7">
+      <c r="G12" s="5">
         <f>+F13*u</f>
         <v>1151.9099101689089</v>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="5">
         <f>+J13*u</f>
         <v>1151.9099101689089</v>
       </c>
@@ -20287,37 +20293,37 @@
         <f>1/B11</f>
         <v>0.86812344539458486</v>
       </c>
-      <c r="F13" s="8">
+      <c r="F13" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="G13" s="12">
+      <c r="G13" s="9">
         <f>+MAX(G12-K,0)</f>
         <v>101.90991016890894</v>
       </c>
-      <c r="J13" s="8">
+      <c r="J13" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="K13" s="12">
+      <c r="K13" s="9">
         <f>+MAX(K-K12,0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F14" s="13">
+      <c r="F14" s="10">
         <f>+MAX((G13*p+G15*q)*EXP(-risk*deltaT),MAX(F13-K,0))</f>
         <v>51.481838003825906</v>
       </c>
-      <c r="G14" s="7">
+      <c r="G14" s="5">
         <f>+F13*d</f>
         <v>868.12344539458491</v>
       </c>
-      <c r="J14" s="13">
+      <c r="J14" s="10">
         <f>+MAX((K13*p+K15*q)*EXP(-risk*deltaT),MAX(K-J13,0))</f>
         <v>85.50741188440719</v>
       </c>
-      <c r="K14" s="7">
+      <c r="K14" s="5">
         <f>+J13*d</f>
         <v>868.12344539458491</v>
       </c>
@@ -20330,11 +20336,11 @@
         <f>+(EXP((risk-rf)*deltaT)-d)/(u-d)</f>
         <v>0.51795852680297783</v>
       </c>
-      <c r="G15" s="12">
+      <c r="G15" s="9">
         <f>+MAX(G14-K,0)</f>
         <v>0</v>
       </c>
-      <c r="K15" s="12">
+      <c r="K15" s="9">
         <f>+MAX(K-K14,0)</f>
         <v>181.87655460541509</v>
       </c>
@@ -20347,34 +20353,34 @@
         <f>1-p</f>
         <v>0.48204147319702217</v>
       </c>
-      <c r="F17" s="6" t="s">
+      <c r="F17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G17" s="6" t="s">
+      <c r="G17" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J17" s="6" t="s">
+      <c r="J17" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K17" s="6" t="s">
+      <c r="K17" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15"/>
+      <c r="D20" s="15"/>
+      <c r="E20" s="15"/>
+      <c r="F20" s="15"/>
+      <c r="G20" s="15"/>
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
@@ -20396,16 +20402,16 @@
         <f>+EXP(vol*SQRT(B21))</f>
         <v>1.1051709180756477</v>
       </c>
-      <c r="F23" s="5" t="s">
+      <c r="F23" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-      <c r="J23" s="5" t="s">
+      <c r="G23" s="16"/>
+      <c r="H23" s="16"/>
+      <c r="J23" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
+      <c r="K23" s="16"/>
+      <c r="L23" s="16"/>
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
@@ -20415,29 +20421,29 @@
         <f>1/B23</f>
         <v>0.90483741803595952</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="5">
         <f>+G26*B23</f>
         <v>1221.4027581601699</v>
       </c>
-      <c r="L25" s="7">
+      <c r="L25" s="5">
         <f>+K26*B23</f>
         <v>1221.4027581601699</v>
       </c>
     </row>
     <row r="26" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="G26" s="7">
+      <c r="G26" s="5">
         <f>+F27*B23</f>
         <v>1105.1709180756477</v>
       </c>
-      <c r="H26" s="12">
+      <c r="H26" s="9">
         <f>+MAX(H25-K,0)</f>
         <v>171.40275816016992</v>
       </c>
-      <c r="K26" s="7">
+      <c r="K26" s="5">
         <f>+J27*B23</f>
         <v>1105.1709180756477</v>
       </c>
-      <c r="L26" s="12">
+      <c r="L26" s="9">
         <f>+MAX(K-L25,0)</f>
         <v>0</v>
       </c>
@@ -20450,53 +20456,53 @@
         <f>+(EXP((risk-rf)*B21)-B25)/(B23-B25)</f>
         <v>0.51259912789538553</v>
       </c>
-      <c r="F27" s="8">
+      <c r="F27" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="G27" s="12">
+      <c r="G27" s="9">
         <f>+MAX((H26*$B$27+H28*$B$29)*EXP(-risk*$B$21),MAX(G26-K,0))</f>
         <v>86.769478669121128</v>
       </c>
-      <c r="H27" s="8">
+      <c r="H27" s="6">
         <f>+G28*B23</f>
         <v>1000.0000000000001</v>
       </c>
-      <c r="J27" s="8">
+      <c r="J27" s="6">
         <f>+S</f>
         <v>1000</v>
       </c>
-      <c r="K27" s="12">
+      <c r="K27" s="9">
         <f>+MAX((L26*$B$27+L28*$B$29)*EXP(-risk*$B$21),MAX(K-K26,0))</f>
         <v>24.067314061593681</v>
       </c>
-      <c r="L27" s="8">
+      <c r="L27" s="6">
         <f>+K28*B23</f>
         <v>1000.0000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F28" s="13">
+      <c r="F28" s="10">
         <f>+MAX((G27*$B$27+G29*$B$29)*EXP(-risk*$B$21),MAX(F27-K,0))</f>
         <v>43.925445012241468</v>
       </c>
-      <c r="G28" s="7">
+      <c r="G28" s="5">
         <f>+F27*B25</f>
         <v>904.83741803595956</v>
       </c>
-      <c r="H28" s="12">
+      <c r="H28" s="9">
         <f>+MAX(H27-K,0)</f>
         <v>0</v>
       </c>
-      <c r="J28" s="13">
+      <c r="J28" s="10">
         <f>+MAX((K27*$B$27+K29*$B$29)*EXP(-risk*$B$21),MAX(K-J27,0))</f>
         <v>82.05710196436452</v>
       </c>
-      <c r="K28" s="7">
+      <c r="K28" s="5">
         <f>+J27*B25</f>
         <v>904.83741803595956</v>
       </c>
-      <c r="L28" s="12">
+      <c r="L28" s="9">
         <f>+MAX(K-L27,0)</f>
         <v>49.999999999999886</v>
       </c>
@@ -20509,96 +20515,96 @@
         <f>1-B27</f>
         <v>0.48740087210461447</v>
       </c>
-      <c r="G29" s="12">
+      <c r="G29" s="9">
         <f>+MAX((H28*$B$27+H30*$B$29)*EXP(-risk*$B$21),MAX(G28-K,0))</f>
         <v>0</v>
       </c>
-      <c r="H29" s="7">
+      <c r="H29" s="5">
         <f>+G28*B25</f>
         <v>818.73075307798183</v>
       </c>
-      <c r="K29" s="12">
+      <c r="K29" s="9">
         <f>+MAX((L28*$B$27+L30*$B$29)*EXP(-risk*$B$21),MAX(K-K28,0))</f>
         <v>145.16258196404044</v>
       </c>
-      <c r="L29" s="7">
+      <c r="L29" s="5">
         <f>+K28*B25</f>
         <v>818.73075307798183</v>
       </c>
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="H30" s="12">
+      <c r="H30" s="9">
         <f>+MAX(H29-K,0)</f>
         <v>0</v>
       </c>
-      <c r="L30" s="12">
+      <c r="L30" s="9">
         <f>+MAX(K-L29,0)</f>
         <v>231.26924692201817</v>
       </c>
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="F32" s="6" t="s">
+      <c r="F32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="G32" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="H32" s="6" t="s">
+      <c r="H32" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="J32" s="6" t="s">
+      <c r="J32" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="K32" s="6" t="s">
+      <c r="K32" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="L32" s="6" t="s">
+      <c r="L32" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="D33" s="9"/>
+      <c r="D33" s="7"/>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A35" s="10" t="s">
+      <c r="A35" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15"/>
+      <c r="L35" s="15"/>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="C37" s="5"/>
-      <c r="D37" s="5"/>
-      <c r="H37" s="5" t="s">
+      <c r="C37" s="16"/>
+      <c r="D37" s="16"/>
+      <c r="H37" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A58" s="10" t="s">
+      <c r="A58" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B58" s="10"/>
-      <c r="C58" s="10"/>
+      <c r="B58" s="15"/>
+      <c r="C58" s="15"/>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B59" s="13">
+      <c r="B59" s="10">
         <v>41.364694755898498</v>
       </c>
     </row>
@@ -20606,7 +20612,7 @@
       <c r="A60" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B60" s="13">
+      <c r="B60" s="10">
         <v>78.076712143941904</v>
       </c>
     </row>
@@ -20653,11 +20659,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:3" ht="17.25" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -20709,7 +20715,7 @@
       </c>
     </row>
     <row r="7" spans="1:3" ht="17.25" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="13" t="s">
         <v>37</v>
       </c>
       <c r="B7" s="3">
@@ -20765,7 +20771,7 @@
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="12">
         <f>+S*EXP(-B7*T/12)*B14-K*EXP(-risk*T/12)*B15</f>
         <v>41.367249386983303</v>
       </c>
@@ -20795,7 +20801,7 @@
       <c r="A23" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B23" s="15">
+      <c r="B23" s="12">
         <f>+K*EXP(-risk*T/12)*B21-S*EXP(-B7*T/12)*B20</f>
         <v>75.392823267564381</v>
       </c>

</xml_diff>

<commit_message>
30 noviembre de 2020 v2
</commit_message>
<xml_diff>
--- a/_downloads/be2fbcfffa0bffb8ba54a662e9d97b81/Ejemplos valoración de opciones por AB y BS.xlsx
+++ b/_downloads/be2fbcfffa0bffb8ba54a662e9d97b81/Ejemplos valoración de opciones por AB y BS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\DERIVADOS FINANCIEROS\CLASES\Opciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5442B786-FBE5-46F0-92AA-2426B5A13303}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E440D59F-020D-4ED9-ADA3-E99BD4E8D989}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{04782C71-9EF5-45E7-9F04-DD1E48186E05}"/>
   </bookViews>
@@ -107,7 +107,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="216" uniqueCount="43">
   <si>
     <t>Volatilidad</t>
   </si>
@@ -372,6 +372,12 @@
   <si>
     <t>Put Americana:</t>
   </si>
+  <si>
+    <t>Call Americana</t>
+  </si>
+  <si>
+    <t>Put Americana</t>
+  </si>
 </sst>
 </file>
 
@@ -6679,7 +6685,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>609599</xdr:colOff>
+      <xdr:colOff>527956</xdr:colOff>
       <xdr:row>55</xdr:row>
       <xdr:rowOff>123314</xdr:rowOff>
     </xdr:to>
@@ -18991,7 +18997,7 @@
   <dimension ref="A1:L60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.42578125" style="1"/>
     <col min="4" max="4" width="10.28515625" style="1" customWidth="1"/>
@@ -19241,12 +19247,12 @@
         <v>1.1051709180756477</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
       <c r="J23" s="16" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="K23" s="16"/>
       <c r="L23" s="16"/>
@@ -19421,12 +19427,12 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B37" s="16" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
       <c r="H37" s="16" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="I37" s="16"/>
       <c r="J37" s="16"/>
@@ -19440,7 +19446,7 @@
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
-        <v>24</v>
+        <v>41</v>
       </c>
       <c r="B59" s="10">
         <v>45.813136870375402</v>
@@ -19448,7 +19454,7 @@
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="B60" s="10">
         <v>74.365645023472894</v>

</xml_diff>

<commit_message>
15 abril de 2021 v1
</commit_message>
<xml_diff>
--- a/_downloads/be2fbcfffa0bffb8ba54a662e9d97b81/Ejemplos valoración de opciones por AB y BS.xlsx
+++ b/_downloads/be2fbcfffa0bffb8ba54a662e9d97b81/Ejemplos valoración de opciones por AB y BS.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23901"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\DERIVADOS FINANCIEROS\CLASES\Opciones\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E440D59F-020D-4ED9-ADA3-E99BD4E8D989}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{496DDE6B-11BE-4581-9569-C9281E1890D1}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{04782C71-9EF5-45E7-9F04-DD1E48186E05}"/>
   </bookViews>
@@ -20409,12 +20409,12 @@
         <v>1.1051709180756477</v>
       </c>
       <c r="F23" s="16" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
       <c r="J23" s="16" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="K23" s="16"/>
       <c r="L23" s="16"/>
@@ -20589,12 +20589,12 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.2">
       <c r="B37" s="16" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
       <c r="H37" s="16" t="s">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="I37" s="16"/>
       <c r="J37" s="16"/>

</xml_diff>